<commit_message>
Nombre directora en Dietas
</commit_message>
<xml_diff>
--- a/backend/DIETAS.xlsx
+++ b/backend/DIETAS.xlsx
@@ -8,10 +8,10 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Anverso" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Reverso" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Autoliquidación" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Instrucciones" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Anverso" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Reverso" sheetId="2" state="visible" r:id="rId3"/>
+    <sheet name="Autoliquidación" sheetId="3" state="visible" r:id="rId4"/>
+    <sheet name="Instrucciones" sheetId="4" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Anverso!$A$1:$R$43</definedName>
@@ -31,15 +31,7 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <authors>
-    <author>BADAJOZ</author>
-    <author>CECT</author>
-    <author>DIRECCION PROVINCIAL BADAJOZ</author>
-    <author>Dirección Provincial Badajoz</author>
-    <author>JOSE LUIS VEGA MORENO</author>
-    <author>Jose Luis Vega</author>
-    <author>José Luis Vega Moreno</author>
-    <author>Juan Jesus Felipe Pizarro</author>
-    <author>cec</author>
+    <author> </author>
   </authors>
   <commentList>
     <comment ref="A8" authorId="0">
@@ -48,19 +40,21 @@
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">CONSIGNAR HORA, DIA Y MES DE  INICIO DE LA COMISIÓN.</t>
         </r>
       </text>
     </comment>
-    <comment ref="A11" authorId="8">
+    <comment ref="A11" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
 SEPARAR HORAS Y MINUTOS CON COMA
@@ -78,13 +72,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="A12" authorId="8">
+    <comment ref="A12" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
 SEPARAR HORAS Y MINUTOS CON COMA
@@ -102,13 +97,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="A13" authorId="8">
+    <comment ref="A13" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
 SEPARAR HORAS Y MINUTOS CON COMA
@@ -126,13 +122,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="A14" authorId="8">
+    <comment ref="A14" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
 SEPARAR HORAS Y MINUTOS CON COMA
@@ -150,13 +147,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="A15" authorId="8">
+    <comment ref="A15" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
 SEPARAR HORAS Y MINUTOS CON COMA
@@ -174,13 +172,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="A16" authorId="8">
+    <comment ref="A16" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
 SEPARAR HORAS Y MINUTOS CON COMA
@@ -198,13 +197,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="A17" authorId="8">
+    <comment ref="A17" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
 SEPARAR HORAS Y MINUTOS CON COMA
@@ -222,13 +222,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="C1" authorId="8">
+    <comment ref="C1" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">cec:
 </t>
@@ -245,13 +246,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="D3" authorId="8">
+    <comment ref="D3" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">cec:
 </t>
@@ -275,19 +277,21 @@
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">EN ESTAS CELDAS FIGURARÁN LOS DATOS RELATIVOS AL REGRESO A LA LOCALIDAD DE PARTIDA, CONSIGNANDO EN "15 horas" UNA "X"  SEGÚN SEA ANTERIOR O POSTERIOR A DICHA HORA. </t>
         </r>
       </text>
     </comment>
-    <comment ref="D9" authorId="5">
+    <comment ref="D9" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">CONSIGNAR UNA X EN ANT. O POST. SEGÚN PROCEDA.
 </t>
@@ -300,111 +304,120 @@
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">CONSIGNAR LAS LOCALIDADES A DONDE SE REALIZA LA COMISIÓN
 </t>
         </r>
       </text>
     </comment>
-    <comment ref="H11" authorId="8">
+    <comment ref="H11" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
 no ponga el origen, sólo la/s localidad/es de DESTINO</t>
         </r>
       </text>
     </comment>
-    <comment ref="H12" authorId="8">
+    <comment ref="H12" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
 no ponga el origen, sólo la/s localidad/es de DESTINO</t>
         </r>
       </text>
     </comment>
-    <comment ref="H13" authorId="8">
+    <comment ref="H13" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
 no ponga el origen, sólo la/s localidad/es de DESTINO</t>
         </r>
       </text>
     </comment>
-    <comment ref="H14" authorId="8">
+    <comment ref="H14" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
 no ponga el origen, sólo la/s localidad/es de DESTINO</t>
         </r>
       </text>
     </comment>
-    <comment ref="H15" authorId="8">
+    <comment ref="H15" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
 no ponga el origen, sólo la/s localidad/es de DESTINO</t>
         </r>
       </text>
     </comment>
-    <comment ref="H16" authorId="8">
+    <comment ref="H16" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
 no ponga el origen, sólo la/s localidad/es de DESTINO</t>
         </r>
       </text>
     </comment>
-    <comment ref="H27" authorId="4">
+    <comment ref="H27" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">LOCALIDAD
 </t>
         </r>
       </text>
     </comment>
-    <comment ref="I39" authorId="3">
+    <comment ref="I39" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">LA FECHA SERÁ IGUAL O POSTERIOR A LA DE LA ÚLTIMA COMISIÓN
 </t>
@@ -422,26 +435,28 @@
         </r>
       </text>
     </comment>
-    <comment ref="J33" authorId="4">
+    <comment ref="J33" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">NOMBRE DEL DIRECTOR DEL CENTRO
 </t>
         </r>
       </text>
     </comment>
-    <comment ref="K27" authorId="4">
+    <comment ref="K27" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">FECHA
 Esta fecha será la misma o anterior a la de la primera comisión.
@@ -449,26 +464,28 @@
         </r>
       </text>
     </comment>
-    <comment ref="L1" authorId="7">
+    <comment ref="L1" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">PARA DESPLAZAMIENTOS DESDE EL 29MAY2025 EN ADELANTE
 </t>
         </r>
       </text>
     </comment>
-    <comment ref="L8" authorId="2">
+    <comment ref="L8" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">CONSIGNAR: 
 </t>
@@ -492,19 +509,21 @@
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">CONSIGNAR  ESCUETAMENTE EL OBJETO DEL VIAJE O COMISIÓN</t>
         </r>
       </text>
     </comment>
-    <comment ref="O4" authorId="8">
+    <comment ref="O4" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">CONSIGNAR  F ó  L
 F  para funcionarios 
@@ -512,13 +531,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="O5" authorId="1">
+    <comment ref="O5" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">CONSIGNAR:
 221-B: C P R
@@ -530,13 +550,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="P3" authorId="6">
+    <comment ref="P3" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">Consignar el porcentaje que a efectos de retención del I.R.P.F. figura en la nómina</t>
         </r>
@@ -549,31 +570,30 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <authors>
-    <author>Dirección Provincial Badajoz</author>
-    <author>JOSE LUIS VEGA MORENO</author>
-    <author>José Luis Vega Moreno</author>
-    <author>cec</author>
+    <author> </author>
   </authors>
   <commentList>
-    <comment ref="A3" authorId="2">
+    <comment ref="A3" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">EL MEDIO DE LOCOMOCIÓN UTILIZADO COINCIDIRÁ CON EL QUE FIGURA EN EL APARTADO "I-PROPUESTA"</t>
         </r>
       </text>
     </comment>
-    <comment ref="A8" authorId="3">
+    <comment ref="A8" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">cec:
 </t>
@@ -591,13 +611,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="A9" authorId="3">
+    <comment ref="A9" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">cec:
 </t>
@@ -615,13 +636,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="A10" authorId="3">
+    <comment ref="A10" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">cec:
 </t>
@@ -639,13 +661,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="A11" authorId="3">
+    <comment ref="A11" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">cec:
 </t>
@@ -663,13 +686,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="A12" authorId="3">
+    <comment ref="A12" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">cec:
 </t>
@@ -687,13 +711,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="A13" authorId="3">
+    <comment ref="A13" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">cec:
 </t>
@@ -711,13 +736,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="A33" authorId="3">
+    <comment ref="A33" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">cec:
 </t>
@@ -734,13 +760,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="D8" authorId="3">
+    <comment ref="D8" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
 SEPARAR HORAS Y MINUTOS CON COMA
@@ -758,13 +785,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="D9" authorId="3">
+    <comment ref="D9" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
 SEPARAR HORAS Y MINUTOS CON COMA
@@ -782,13 +810,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="D10" authorId="3">
+    <comment ref="D10" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
 SEPARAR HORAS Y MINUTOS CON COMA
@@ -806,13 +835,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="D11" authorId="3">
+    <comment ref="D11" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
 SEPARAR HORAS Y MINUTOS CON COMA
@@ -830,13 +860,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="D12" authorId="3">
+    <comment ref="D12" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
 SEPARAR HORAS Y MINUTOS CON COMA
@@ -854,13 +885,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="D13" authorId="3">
+    <comment ref="D13" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
 SEPARAR HORAS Y MINUTOS CON COMA
@@ -884,7 +916,8 @@
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">NOMBRE DEL DECLARANTE.</t>
         </r>
@@ -896,20 +929,22 @@
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">LA FECHA DEBE SER IGUAL O POSTERIOR A LA DE LA ÚLTIMA COMISIÓN
 </t>
         </r>
       </text>
     </comment>
-    <comment ref="J50" authorId="1">
+    <comment ref="J50" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">NOMBRE DEL DECLARANTE.</t>
         </r>
@@ -922,18 +957,17 @@
 <file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <authors>
-    <author>Jose Luis Vega</author>
-    <author>Juan Jesus Felipe Pizarro</author>
-    <author>cec</author>
+    <author> </author>
   </authors>
   <commentList>
-    <comment ref="D12" authorId="1">
+    <comment ref="D12" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
 Cruzo la frontera, como o ceno y me vuelvo.
@@ -941,13 +975,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="D14" authorId="2">
+    <comment ref="D14" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">MAXIMO PERMITIDO:   UNA
 Sólo para el día de ida, </t>
@@ -965,25 +1000,27 @@
         </r>
       </text>
     </comment>
-    <comment ref="D16" authorId="1">
+    <comment ref="D16" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">Una vez cruzada la frontera, como y ceno y me vuelvo a casa</t>
         </r>
       </text>
     </comment>
-    <comment ref="E22" authorId="2">
+    <comment ref="E22" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">IMPORTE PAGADO POR ALOJAMIENTO Y DESAYUNO  
 La factura de hotel (obligatoria) se acompañará cuando se presenten los impresos del desplazamiento.
@@ -991,13 +1028,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="E23" authorId="2">
+    <comment ref="E23" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">IMPORTE PAGADO POR ALOJAMIENTO Y DESAYUNO  
 La factura/s de hotel (obligatoria) se acompañará cuando se presenten los impresos del desplazamiento.
@@ -1005,13 +1043,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="E25" authorId="2">
+    <comment ref="E25" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">IMPORTE PAGADO POR ALOJAMIENTO Y DESAYUNO  
 La factura/s de hotel (obligatoria) se acompañará cuando se presenten los impresos del desplazamiento.
@@ -1019,13 +1058,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="G15" authorId="2">
+    <comment ref="G15" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">MAXIMO PERMITIDO:   UNA
 </t>
@@ -1043,13 +1083,14 @@
         </r>
       </text>
     </comment>
-    <comment ref="G17" authorId="1">
+    <comment ref="G17" authorId="0">
       <text>
         <r>
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">Salgo del termino municipal del colegio o de mi casa,  como y ceno y vuelvo.</t>
         </r>
@@ -1061,7 +1102,8 @@
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">IMPORTE ABONADO 
 </t>
@@ -1085,7 +1127,8 @@
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">IMPORTE ABONADO
 </t>
@@ -1109,7 +1152,8 @@
           <rPr>
             <sz val="10"/>
             <rFont val="Arial"/>
-            <family val="2"/>
+            <family val="0"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">IMPORTE ABONADO
 </t>
@@ -1261,7 +1305,7 @@
     <t xml:space="preserve">Fdo.:</t>
   </si>
   <si>
-    <t xml:space="preserve">MARÍA MONTAÑA HERNÁNDEZ GIL</t>
+    <t xml:space="preserve">MARÍA MONTAÑA HERNÁNDEZ ROSADO</t>
   </si>
   <si>
     <t xml:space="preserve">III.- CERTIFICADO REALIZACIÓN DE LA COMISIÓN:</t>
@@ -2596,7 +2640,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="14">
+  <numFmts count="15">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0;[RED]#,##0;#"/>
     <numFmt numFmtId="166" formatCode="0.00"/>
@@ -2607,12 +2651,13 @@
     <numFmt numFmtId="171" formatCode="#,##0.00;[RED]#,##0.00;#"/>
     <numFmt numFmtId="172" formatCode="0;[RED]0"/>
     <numFmt numFmtId="173" formatCode="#,##0.00&quot; €&quot;;[RED]#,##0.00&quot; €&quot;;#"/>
-    <numFmt numFmtId="174" formatCode="#,##0.00&quot; €&quot;"/>
-    <numFmt numFmtId="175" formatCode="#,##0.00&quot; %&quot;"/>
-    <numFmt numFmtId="176" formatCode="_-* #,##0.00&quot; €&quot;_-;\-* #,##0.00&quot; €&quot;_-;_-* \-??&quot; €&quot;_-;_-@_-"/>
-    <numFmt numFmtId="177" formatCode="#,##0"/>
+    <numFmt numFmtId="174" formatCode="General"/>
+    <numFmt numFmtId="175" formatCode="#,##0.00&quot; €&quot;"/>
+    <numFmt numFmtId="176" formatCode="#,##0.00&quot; %&quot;"/>
+    <numFmt numFmtId="177" formatCode="_-* #,##0.00&quot; €&quot;_-;\-* #,##0.00&quot; €&quot;_-;_-* \-??&quot; €&quot;_-;_-@_-"/>
+    <numFmt numFmtId="178" formatCode="#,##0"/>
   </numFmts>
-  <fonts count="36">
+  <fonts count="35">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -2693,11 +2738,6 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
@@ -2878,13 +2918,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="2" tint="-0.1"/>
+        <fgColor rgb="FFD0CECE"/>
         <bgColor rgb="FFC0C0C0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="2" tint="-0.25"/>
+        <fgColor rgb="FFAFABAB"/>
         <bgColor rgb="FFA0B0C0"/>
       </patternFill>
     </fill>
@@ -3669,7 +3709,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
@@ -4216,15 +4256,15 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="17" fillId="0" borderId="54" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="171" fontId="16" fillId="0" borderId="54" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="17" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="171" fontId="16" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="17" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="171" fontId="16" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4340,7 +4380,7 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="18" fillId="2" borderId="71" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="173" fontId="17" fillId="2" borderId="71" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="true"/>
     </xf>
@@ -4352,7 +4392,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="73" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="174" fontId="0" fillId="2" borderId="73" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4368,11 +4408,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="18" fillId="2" borderId="72" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="17" fillId="2" borderId="72" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="2" borderId="71" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="174" fontId="17" fillId="2" borderId="71" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="true"/>
     </xf>
@@ -4392,55 +4432,55 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="3" borderId="77" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="19" fillId="3" borderId="77" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="2" borderId="78" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="21" fillId="2" borderId="78" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="2" borderId="79" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="23" fillId="2" borderId="80" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="174" fontId="22" fillId="2" borderId="79" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="22" fillId="2" borderId="80" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="2" borderId="80" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="23" fillId="2" borderId="80" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="170" fontId="22" fillId="2" borderId="80" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="2" borderId="81" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="21" fillId="2" borderId="81" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="23" fillId="3" borderId="82" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="22" fillId="3" borderId="82" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="23" fillId="3" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="22" fillId="3" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="23" fillId="3" borderId="83" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="22" fillId="3" borderId="83" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="23" fillId="0" borderId="84" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="22" fillId="0" borderId="84" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4448,83 +4488,295 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="true"/>
     </xf>
-    <xf numFmtId="174" fontId="24" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="175" fontId="23" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="true"/>
     </xf>
-    <xf numFmtId="175" fontId="24" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="176" fontId="23" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="true"/>
     </xf>
-    <xf numFmtId="174" fontId="24" fillId="0" borderId="85" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="175" fontId="23" fillId="0" borderId="85" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="true"/>
     </xf>
-    <xf numFmtId="165" fontId="23" fillId="0" borderId="86" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="22" fillId="0" borderId="86" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="24" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="175" fontId="23" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="24" fillId="0" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="23" fillId="0" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="true"/>
     </xf>
-    <xf numFmtId="175" fontId="24" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="176" fontId="23" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="true"/>
     </xf>
-    <xf numFmtId="173" fontId="24" fillId="0" borderId="87" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="173" fontId="23" fillId="0" borderId="87" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="true"/>
     </xf>
-    <xf numFmtId="173" fontId="24" fillId="0" borderId="85" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="173" fontId="23" fillId="0" borderId="85" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="true"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="24" fillId="0" borderId="88" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="23" fillId="0" borderId="88" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="true"/>
     </xf>
-    <xf numFmtId="175" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="176" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="true"/>
     </xf>
-    <xf numFmtId="173" fontId="24" fillId="0" borderId="72" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="173" fontId="23" fillId="0" borderId="72" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="true"/>
     </xf>
-    <xf numFmtId="166" fontId="24" fillId="0" borderId="89" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="23" fillId="0" borderId="89" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="true"/>
     </xf>
-    <xf numFmtId="175" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="176" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="true"/>
     </xf>
-    <xf numFmtId="173" fontId="24" fillId="0" borderId="90" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="173" fontId="23" fillId="0" borderId="90" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="true"/>
     </xf>
-    <xf numFmtId="165" fontId="25" fillId="2" borderId="91" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="24" fillId="2" borderId="91" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="26" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="175" fontId="25" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="true"/>
+    </xf>
+    <xf numFmtId="176" fontId="25" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="true"/>
+    </xf>
+    <xf numFmtId="175" fontId="25" fillId="0" borderId="11" xfId="17" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="true"/>
+    </xf>
+    <xf numFmtId="175" fontId="25" fillId="0" borderId="85" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="true"/>
+    </xf>
+    <xf numFmtId="165" fontId="21" fillId="0" borderId="86" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="92" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="26" fillId="3" borderId="93" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="27" fillId="4" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="3" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="22" fillId="3" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="22" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="22" fillId="3" borderId="94" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="22" fillId="0" borderId="95" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="96" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="175" fontId="23" fillId="0" borderId="96" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="5" borderId="87" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="176" fontId="21" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="true"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="5" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="178" fontId="23" fillId="0" borderId="87" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="175" fontId="23" fillId="0" borderId="87" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="87" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="23" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="175" fontId="23" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="23" fillId="0" borderId="96" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="24" fillId="2" borderId="97" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="25" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="true"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="86" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="3" borderId="93" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="22" fillId="6" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="82" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="175" fontId="23" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="175" fontId="23" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="25" fillId="0" borderId="85" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="true"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="95" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="96" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="23" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="27" fillId="0" borderId="82" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="82" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="25" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="175" fontId="25" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="24" fillId="2" borderId="98" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="25" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="25" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="25" fillId="2" borderId="99" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="23" fillId="3" borderId="86" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="3" borderId="92" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="28" fillId="3" borderId="86" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="72" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="26" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="true"/>
     </xf>
@@ -4532,259 +4784,47 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="true"/>
     </xf>
-    <xf numFmtId="174" fontId="26" fillId="0" borderId="11" xfId="17" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="true"/>
-    </xf>
-    <xf numFmtId="174" fontId="26" fillId="0" borderId="85" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="true"/>
-    </xf>
-    <xf numFmtId="165" fontId="22" fillId="0" borderId="86" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="92" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="27" fillId="3" borderId="93" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="28" fillId="4" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="23" fillId="3" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="23" fillId="3" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="23" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="23" fillId="3" borderId="94" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="23" fillId="0" borderId="95" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="96" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="174" fontId="24" fillId="0" borderId="96" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="24" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="false" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="24" fillId="5" borderId="87" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="175" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="true"/>
-    </xf>
-    <xf numFmtId="164" fontId="24" fillId="5" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="177" fontId="24" fillId="0" borderId="87" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="false" hidden="false"/>
-    </xf>
-    <xf numFmtId="174" fontId="24" fillId="0" borderId="87" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="24" fillId="0" borderId="87" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="false" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="24" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="false" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="174" fontId="24" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="24" fillId="0" borderId="96" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="false" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="25" fillId="2" borderId="97" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="26" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="true"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="86" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="23" fillId="3" borderId="93" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="23" fillId="6" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="82" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="174" fontId="24" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="false" hidden="false"/>
-    </xf>
-    <xf numFmtId="174" fontId="24" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="173" fontId="26" fillId="0" borderId="85" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="true"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="95" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="21" fillId="3" borderId="100" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="3" borderId="77" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="3" borderId="101" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="96" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="24" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="28" fillId="0" borderId="82" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="false" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="82" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="26" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="174" fontId="26" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="25" fillId="2" borderId="98" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="26" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="173" fontId="26" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="173" fontId="26" fillId="2" borderId="99" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="24" fillId="3" borderId="86" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="23" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="23" fillId="3" borderId="92" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="29" fillId="3" borderId="86" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="72" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="173" fontId="27" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="true"/>
-    </xf>
-    <xf numFmtId="174" fontId="27" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="true"/>
-    </xf>
-    <xf numFmtId="173" fontId="27" fillId="0" borderId="85" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="true"/>
-    </xf>
-    <xf numFmtId="165" fontId="22" fillId="3" borderId="100" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="3" borderId="77" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="3" borderId="101" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="30" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="29" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="30" fillId="2" borderId="102" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="29" fillId="2" borderId="102" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="31" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="30" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="31" fillId="2" borderId="103" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="30" fillId="2" borderId="103" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="31" fillId="2" borderId="104" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="30" fillId="2" borderId="104" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4824,11 +4864,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4957,14 +4997,14 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="7" tint="0.3999"/>
+          <bgColor rgb="FFFFD966"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="7" tint="0.5999"/>
+          <bgColor rgb="FFFFE699"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5041,7 +5081,7 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:twoCellAnchor editAs="twoCell">
+  <xdr:twoCellAnchor editAs="absolute">
     <xdr:from>
       <xdr:col>13</xdr:col>
       <xdr:colOff>152280</xdr:colOff>
@@ -5050,75 +5090,75 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>20</xdr:col>
-      <xdr:colOff>94320</xdr:colOff>
+      <xdr:colOff>93960</xdr:colOff>
       <xdr:row>27</xdr:row>
-      <xdr:rowOff>84960</xdr:rowOff>
+      <xdr:rowOff>84600</xdr:rowOff>
     </xdr:to>
-    <xdr:grpSp>
-      <xdr:nvGrpSpPr>
-        <xdr:cNvPr id="0" name="Grupo 6"/>
-        <xdr:cNvGrpSpPr/>
-      </xdr:nvGrpSpPr>
-      <xdr:grpSpPr>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="Imagen 1" descr=""/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
         <a:xfrm>
-          <a:off x="10119240" y="190440"/>
-          <a:ext cx="5578200" cy="6304680"/>
-          <a:chOff x="10119240" y="190440"/>
-          <a:chExt cx="5578200" cy="6304680"/>
+          <a:off x="10128240" y="190440"/>
+          <a:ext cx="5586840" cy="6304320"/>
         </a:xfrm>
-      </xdr:grpSpPr>
-      <xdr:pic>
-        <xdr:nvPicPr>
-          <xdr:cNvPr id="1" name="Imagen 1" descr=""/>
-          <xdr:cNvPicPr/>
-        </xdr:nvPicPr>
-        <xdr:blipFill>
-          <a:blip r:embed="rId1"/>
-          <a:stretch/>
-        </xdr:blipFill>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="10119240" y="190440"/>
-            <a:ext cx="5578200" cy="6304680"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
           <a:noFill/>
-          <a:ln w="0">
-            <a:noFill/>
-          </a:ln>
-        </xdr:spPr>
-      </xdr:pic>
-      <xdr:sp>
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="2" name="Elipse 5"/>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="13623120" y="2705400"/>
-            <a:ext cx="876600" cy="252000"/>
-          </a:xfrm>
-          <a:prstGeom prst="ellipse">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-          <a:ln w="28575">
-            <a:solidFill>
-              <a:srgbClr val="00b050"/>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-        </xdr:spPr>
-        <xdr:style>
-          <a:lnRef idx="0"/>
-          <a:fillRef idx="0"/>
-          <a:effectRef idx="0"/>
-          <a:fontRef idx="minor"/>
-        </xdr:style>
-      </xdr:sp>
-    </xdr:grpSp>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="absolute">
+    <xdr:from>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>436320</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>133560</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>507600</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>137520</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1" name="Elipse 5"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="13637880" y="2705400"/>
+          <a:ext cx="877680" cy="251640"/>
+        </a:xfrm>
+        <a:prstGeom prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="28575">
+          <a:solidFill>
+            <a:srgbClr val="00b050"/>
+          </a:solidFill>
+          <a:round/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0"/>
+        <a:fillRef idx="0"/>
+        <a:effectRef idx="0"/>
+        <a:fontRef idx="minor"/>
+      </xdr:style>
+    </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
@@ -5130,13 +5170,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>27</xdr:col>
-      <xdr:colOff>98280</xdr:colOff>
+      <xdr:colOff>97920</xdr:colOff>
       <xdr:row>29</xdr:row>
-      <xdr:rowOff>100440</xdr:rowOff>
+      <xdr:rowOff>100080</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Imagen 7" descr=""/>
+        <xdr:cNvPr id="2" name="Imagen 7" descr=""/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -5145,13 +5185,12 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="16408440" y="361800"/>
-          <a:ext cx="4929480" cy="6463440"/>
+          <a:off x="16427520" y="361800"/>
+          <a:ext cx="4936680" cy="6463080"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:noFill/>
         <a:ln w="0">
           <a:noFill/>
         </a:ln>
@@ -5162,198 +5201,26 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tema de Office">
-  <a:themeElements>
-    <a:clrScheme name="Office">
-      <a:dk1>
-        <a:srgbClr val="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:srgbClr val="ffffff"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="44546a"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="e7e6e6"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="5b9bd5"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="ed7d31"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="a5a5a5"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="ffc000"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="4472c4"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="70ad47"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="0563c1"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="954f72"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204" pitchFamily="0" charset="1"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="0" charset="1"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme>
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:tint val="67000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:tint val="73000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:tint val="81000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:shade val="78000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-</a:theme>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:R1048"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.43359375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="4.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="3.99"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="3.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="3.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="4.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="6.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="6.42"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="11.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="17.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="17.58"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="11.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="10.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="7.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="10.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="7.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="11.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="12.71"/>
@@ -5974,7 +5841,7 @@
       <c r="J27" s="66"/>
       <c r="K27" s="67" t="str">
         <f aca="true">CONCATENATE("  a     ",B11,"  de        ",IF(C11=1,"Enero",IF(C11=2,"Febrero",IF(C11=3,"Marzo",IF(C11=4,"Abril",IF(C11=5,"Mayo",IF(C11=6,"Junio",IF(C11=9,"Septiembre",""))))))),IF(C11=10,"Octubre",IF(C11=11,"Noviembre",IF(C11=12,"Diciembre","")))," de   ",IF(AND(C11=12,MONTH(TODAY())=1),YEAR(TODAY())-1,YEAR(TODAY())))</f>
-        <v>  a       de         de   2025</v>
+        <v>  a       de         de   2026</v>
       </c>
       <c r="L27" s="67"/>
       <c r="M27" s="67"/>
@@ -6104,7 +5971,7 @@
       <c r="H39" s="70"/>
       <c r="I39" s="75" t="str">
         <f aca="false">Reverso!I24</f>
-        <v>0 / 0 / 2025</v>
+        <v>0 / 0 / 2026</v>
       </c>
       <c r="J39" s="75"/>
     </row>
@@ -6112,7 +5979,7 @@
     <row r="43" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H43" s="66" t="str">
         <f aca="false">J33</f>
-        <v>MARÍA MONTAÑA HERNÁNDEZ GIL</v>
+        <v>MARÍA MONTAÑA HERNÁNDEZ ROSADO</v>
       </c>
       <c r="I43" s="66"/>
       <c r="J43" s="66"/>
@@ -26209,15 +26076,15 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:S51"/>
-  <sheetFormatPr defaultColWidth="11.43359375" defaultRowHeight="12.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.4453125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="77" width="4.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="77" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="77" width="6.01"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="77" width="4.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="77" width="5.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="77" width="9"/>
@@ -26228,11 +26095,11 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="77" width="4.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="77" width="4.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="77" width="5.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="15" style="77" width="5.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="15" style="77" width="5.7"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="17" min="17" style="78" width="11.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="78" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="78" width="10.99"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="77" width="9.42"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="20" style="77" width="11.43"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="20" style="77" width="11.43"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -26980,7 +26847,7 @@
       </c>
       <c r="I24" s="114" t="str">
         <f aca="true">CONCATENATE(MAX(E8:E22)," / ",MAX(F8:F22)," / ",IF(AND(MAX(F8:F22)=12,MONTH(TODAY())=1),YEAR(TODAY())-1,YEAR(TODAY())))</f>
-        <v>0 / 0 / 2025</v>
+        <v>0 / 0 / 2026</v>
       </c>
       <c r="J24" s="114"/>
       <c r="K24" s="114"/>
@@ -27590,7 +27457,7 @@
       <c r="D50" s="176"/>
       <c r="E50" s="177" t="str">
         <f aca="false">IF(Anverso!J33&lt;&gt;"","Fdo.:"&amp;Anverso!J33,"")</f>
-        <v>Fdo.:MARÍA MONTAÑA HERNÁNDEZ GIL</v>
+        <v>Fdo.:MARÍA MONTAÑA HERNÁNDEZ ROSADO</v>
       </c>
       <c r="F50" s="177"/>
       <c r="G50" s="177"/>
@@ -27728,24 +27595,24 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:Q135"/>
-  <sheetFormatPr defaultColWidth="11.43359375" defaultRowHeight="12.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.4453125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="179" width="19.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="179" width="19.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="179" width="11.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="179" width="12.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="179" width="3.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="179" width="3.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="179" width="2.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="179" width="9.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="179" width="13.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="179" width="9.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="179" width="13.7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="179" width="10.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="179" width="13.71"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="70" style="179" width="11.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="179" width="13.7"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="70" style="179" width="11.43"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27784,7 +27651,7 @@
       </c>
       <c r="J2" s="185" t="str">
         <f aca="false">IF(Reverso!I24&lt;&gt;"",Reverso!I24,"")</f>
-        <v>0 / 0 / 2025</v>
+        <v>0 / 0 / 2026</v>
       </c>
       <c r="K2" s="185"/>
       <c r="L2" s="185"/>
@@ -29760,12 +29627,12 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:F50"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.43359375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="76" width="79.57"/>
   </cols>

</xml_diff>